<commit_message>
Update latest learning hub changes
</commit_message>
<xml_diff>
--- a/public/data/raw/Pilots.xlsx
+++ b/public/data/raw/Pilots.xlsx
@@ -1,12 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Arif Iqbal\elite-elearning-platform\elite-elearning-platform\public\data\raw\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BEDCEE7-3537-47F8-9E2F-4B47FDAC1709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$24</definedName>
+  </definedNames>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -109,16 +121,16 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="&quot;Aptos Narrow&quot;"/>
     </font>
@@ -128,35 +140,39 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -164,7 +180,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -354,17 +370,23 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:E24"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col min="3" max="3" width="99" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:5" ht="14.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -377,13 +399,14 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2">
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="14.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2">
-        <v>1.0</v>
+      <c r="B2">
+        <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>5</v>
@@ -392,12 +415,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:5" ht="14.25">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="2">
-        <v>2.0</v>
+      <c r="B3">
+        <v>17</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>8</v>
@@ -406,12 +429,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:5" ht="14.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2">
-        <v>3.0</v>
+      <c r="B4">
+        <v>7</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>9</v>
@@ -420,12 +443,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:5" ht="14.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2">
-        <v>4.0</v>
+      <c r="B5">
+        <v>8</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>10</v>
@@ -434,12 +457,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:5" ht="14.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="2">
-        <v>5.0</v>
+      <c r="B6">
+        <v>9</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>11</v>
@@ -448,12 +471,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:5" ht="14.25">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="2">
-        <v>6.0</v>
+      <c r="B7">
+        <v>10</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>12</v>
@@ -462,12 +485,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:5" ht="14.25">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="2">
-        <v>7.0</v>
+      <c r="B8">
+        <v>11</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>13</v>
@@ -476,12 +499,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:5" ht="14.25">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="2">
-        <v>8.0</v>
+      <c r="B9">
+        <v>12</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>14</v>
@@ -490,12 +513,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:5" ht="14.25">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="2">
-        <v>9.0</v>
+      <c r="B10">
+        <v>13</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>15</v>
@@ -504,12 +527,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:5" ht="14.25">
       <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="2">
-        <v>10.0</v>
+      <c r="B11">
+        <v>14</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>16</v>
@@ -518,12 +541,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:5" ht="14.25">
       <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="2">
-        <v>11.0</v>
+      <c r="B12">
+        <v>15</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>18</v>
@@ -532,12 +555,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:5" ht="14.25">
       <c r="A13" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="2">
-        <v>12.0</v>
+      <c r="B13">
+        <v>16</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>19</v>
@@ -546,12 +569,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:5" ht="14.25">
       <c r="A14" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="2">
-        <v>13.0</v>
+      <c r="B14">
+        <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>20</v>
@@ -560,12 +583,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:5" ht="14.25">
       <c r="A15" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="2">
-        <v>14.0</v>
+      <c r="B15">
+        <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>21</v>
@@ -574,12 +597,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:5" ht="14.25">
       <c r="A16" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="2">
-        <v>15.0</v>
+      <c r="B16">
+        <v>3</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>22</v>
@@ -588,12 +611,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:4" ht="14.25">
       <c r="A17" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B17" s="2">
-        <v>16.0</v>
+      <c r="B17">
+        <v>19</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>23</v>
@@ -602,12 +625,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:4" ht="14.25">
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="2">
-        <v>17.0</v>
+      <c r="B18">
+        <v>20</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>24</v>
@@ -616,12 +639,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:4" ht="14.25">
       <c r="A19" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="2">
-        <v>18.0</v>
+      <c r="B19">
+        <v>21</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>25</v>
@@ -630,12 +653,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:4" ht="14.25">
       <c r="A20" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B20" s="2">
-        <v>19.0</v>
+      <c r="B20">
+        <v>22</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>26</v>
@@ -644,12 +667,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:4" ht="14.25">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="2">
-        <v>20.0</v>
+      <c r="B21">
+        <v>23</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>27</v>
@@ -658,12 +681,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:4" ht="14.25">
       <c r="A22" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B22" s="2">
-        <v>21.0</v>
+      <c r="B22">
+        <v>24</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>28</v>
@@ -672,12 +695,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:4" ht="14.25">
       <c r="A23" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B23" s="2">
-        <v>22.0</v>
+      <c r="B23">
+        <v>25</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>29</v>
@@ -686,12 +709,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:4" ht="14.25">
       <c r="A24" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B24" s="2">
-        <v>23.0</v>
+      <c r="B24">
+        <v>26</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>30</v>
@@ -701,6 +724,6 @@
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>